<commit_message>
Update June time tracking workbook
</commit_message>
<xml_diff>
--- a/outputs/time_tracking_taetigkeitsschein/CMC_Time_Tracking_Taetigkeitsschein_Juni_2026.xlsx
+++ b/outputs/time_tracking_taetigkeitsschein/CMC_Time_Tracking_Taetigkeitsschein_Juni_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mariaake/Documents/CMC/outputs/time_tracking_taetigkeitsschein/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{726E9633-7BA8-474A-8377-7B9B7E977C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E02D864B-ABC8-C34B-8B54-DABEAB8BB5FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8880" yWindow="1800" windowWidth="29400" windowHeight="16660" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="269">
   <si>
     <t>Datenbasis</t>
   </si>
@@ -843,6 +843,12 @@
   </si>
   <si>
     <t>Abfrage Produktgruppen bei Yonne, Antwort Christina, Zusammenfassung Short.io + Nachfrage Short.io zu den letzten offenen Fragen + erneute Antwort von Shortio an Robert geben</t>
+  </si>
+  <si>
+    <t>Daily + Pre-Test und letzte Punkte zur Übergabe</t>
+  </si>
+  <si>
+    <t>Voraussichtlich: Weekly Meeting Deutsche Post + Nacharbeiten</t>
   </si>
 </sst>
 </file>
@@ -2852,7 +2858,7 @@
       </c>
       <c r="B14" s="41">
         <f>SUMIFS(Datenbasis!$E$13:$E$214,Datenbasis!$A$13:$A$214,"&gt;="&amp;A14,Datenbasis!$A$13:$A$214,"&lt;"&amp;EDATE(A14,1))</f>
-        <v>59.55</v>
+        <v>61.55</v>
       </c>
       <c r="C14" s="41">
         <f>SUMIFS(Datenbasis!$L$13:$L$214,Datenbasis!$A$13:$A$214,"&gt;="&amp;A14,Datenbasis!$A$13:$A$214,"&lt;"&amp;EDATE(A14,1))</f>
@@ -2860,7 +2866,7 @@
       </c>
       <c r="D14" s="42">
         <f>SUMIFS(Datenbasis!$M$13:$M$214,Datenbasis!$A$13:$A$214,"&gt;="&amp;A14,Datenbasis!$A$13:$A$214,"&lt;"&amp;EDATE(A14,1))</f>
-        <v>2.5499999999999972</v>
+        <v>4.5499999999999972</v>
       </c>
       <c r="E14" s="42" t="str">
         <f>IF(Einstellungen!$B$14="","",Einstellungen!$B$14)</f>
@@ -4005,7 +4011,7 @@
       </c>
       <c r="B51" s="41">
         <f>IF(SUMIFS(Datenbasis!$E$13:$E$214,Datenbasis!$H$13:$H$214,A51)=0,"",SUMIFS(Datenbasis!$E$13:$E$214,Datenbasis!$H$13:$H$214,A51))</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C51" s="41">
         <f>IF(B51="","",SUMIFS(Datenbasis!$L$13:$L$214,Datenbasis!$H$13:$H$214,A51))</f>
@@ -4013,7 +4019,7 @@
       </c>
       <c r="D51" s="42">
         <f>IF(B51="","",SUMIFS(Datenbasis!$M$13:$M$214,Datenbasis!$H$13:$H$214,A51))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E51" s="42">
         <f>IF(OR(B51="",Einstellungen!$B$15=""),"",Einstellungen!$B$15)</f>
@@ -5172,7 +5178,7 @@
       </c>
       <c r="I5" s="52">
         <f ca="1">SUMIFS($E$13:$E$214,$A$13:$A$214,"&gt;="&amp;$H$5,$A$13:$A$214,"&lt;"&amp;$H$5+7)</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J5" s="53">
         <f>Einstellungen!$B$15</f>
@@ -5180,7 +5186,7 @@
       </c>
       <c r="K5" s="52">
         <f ca="1">IF(OR(I5="",J5=""),"",J5-I5)</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="15" customHeight="1">
@@ -7988,11 +7994,11 @@
       </c>
       <c r="N65" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O65" s="59">
         <f>IF(A65="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N65))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="66" spans="1:15" s="57" customFormat="1" ht="54" customHeight="1">
@@ -8034,11 +8040,11 @@
       </c>
       <c r="N66" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O66" s="59">
         <f>IF(A66="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N66))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="67" spans="1:15" ht="54" customHeight="1">
@@ -8083,11 +8089,11 @@
       </c>
       <c r="N67" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O67" s="59">
         <f>IF(A67="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N67))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="68" spans="1:15" ht="54" customHeight="1">
@@ -8132,11 +8138,11 @@
       </c>
       <c r="N68" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O68" s="59">
         <f>IF(A68="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N68))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="69" spans="1:15" ht="54" customHeight="1">
@@ -8181,11 +8187,11 @@
       </c>
       <c r="N69" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O69" s="59">
         <f>IF(A69="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N69))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="70" spans="1:15" ht="54" customHeight="1">
@@ -8230,11 +8236,11 @@
       </c>
       <c r="N70" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O70" s="59">
         <f>IF(A70="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N70))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="71" spans="1:15" ht="54" customHeight="1">
@@ -8279,11 +8285,11 @@
       </c>
       <c r="N71" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O71" s="59">
         <f>IF(A71="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N71))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="72" spans="1:15" ht="54" customHeight="1">
@@ -8328,11 +8334,11 @@
       </c>
       <c r="N72" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O72" s="59">
         <f>IF(A72="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N72))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="73" spans="1:15" ht="54" customHeight="1">
@@ -8377,11 +8383,11 @@
       </c>
       <c r="N73" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O73" s="59">
         <f>IF(A73="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N73))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="74" spans="1:15" ht="54" customHeight="1">
@@ -8426,11 +8432,11 @@
       </c>
       <c r="N74" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O74" s="59">
         <f>IF(A74="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N74))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="75" spans="1:15" ht="54" customHeight="1">
@@ -8475,11 +8481,11 @@
       </c>
       <c r="N75" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O75" s="59">
         <f>IF(A75="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N75))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="76" spans="1:15" ht="54" customHeight="1">
@@ -8524,11 +8530,11 @@
       </c>
       <c r="N76" s="59">
         <f t="shared" si="4"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O76" s="59">
         <f>IF(A76="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N76))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="77" spans="1:15" ht="54" customHeight="1">
@@ -8573,11 +8579,11 @@
       </c>
       <c r="N77" s="59">
         <f t="shared" ref="N77:N140" si="10">IF(A77="","",SUMIFS($E$13:$E$214,$H$13:$H$214,H77))</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O77" s="59">
         <f>IF(A77="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N77))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="78" spans="1:15" ht="54" customHeight="1">
@@ -8622,11 +8628,11 @@
       </c>
       <c r="N78" s="59">
         <f t="shared" si="10"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O78" s="59">
         <f>IF(A78="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N78))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="79" spans="1:15" ht="54" customHeight="1">
@@ -8671,11 +8677,11 @@
       </c>
       <c r="N79" s="59">
         <f t="shared" si="10"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O79" s="59">
         <f>IF(A79="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N79))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="80" spans="1:15" ht="54" customHeight="1">
@@ -8720,11 +8726,11 @@
       </c>
       <c r="N80" s="59">
         <f t="shared" si="10"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O80" s="59">
         <f>IF(A80="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N80))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="81" spans="1:15" ht="54" customHeight="1">
@@ -8769,11 +8775,11 @@
       </c>
       <c r="N81" s="59">
         <f t="shared" si="10"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O81" s="59">
         <f>IF(A81="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N81))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="82" spans="1:15" ht="54" customHeight="1">
@@ -8818,93 +8824,109 @@
       </c>
       <c r="N82" s="59">
         <f t="shared" si="10"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="O82" s="59">
         <f>IF(A82="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N82))</f>
-        <v>-1</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="83" spans="1:15" ht="54" customHeight="1">
-      <c r="A83" s="54"/>
-      <c r="B83" s="13"/>
+      <c r="A83" s="54">
+        <v>46218</v>
+      </c>
+      <c r="B83" s="13" t="s">
+        <v>50</v>
+      </c>
       <c r="C83" s="13"/>
-      <c r="D83" s="13"/>
-      <c r="E83" s="46"/>
-      <c r="F83" s="46" t="str">
+      <c r="D83" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="E83" s="46">
+        <v>0.75</v>
+      </c>
+      <c r="F83" s="46">
         <f>IF(A83="","",Einstellungen!$B$5)</f>
-        <v/>
-      </c>
-      <c r="G83" s="47" t="str">
+        <v>85</v>
+      </c>
+      <c r="G83" s="47">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H83" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="H83" s="14">
         <f t="shared" si="8"/>
-        <v/>
+        <v>29</v>
       </c>
       <c r="I83" s="13" t="str">
         <f t="shared" si="6"/>
-        <v/>
+        <v>Juli YYYY</v>
       </c>
       <c r="J83" s="13"/>
       <c r="K83" s="13"/>
-      <c r="L83" s="59" t="str">
+      <c r="L83" s="59">
         <f>IF(A83="","",IF(Einstellungen!$B$15="","",MAX(0,MIN(E83,Einstellungen!$B$15-(SUMIFS($E$13:$E83,$H$13:$H83,H83)-E83)))))</f>
-        <v/>
-      </c>
-      <c r="M83" s="59" t="str">
+        <v>0</v>
+      </c>
+      <c r="M83" s="59">
         <f t="shared" si="9"/>
-        <v/>
-      </c>
-      <c r="N83" s="59" t="str">
+        <v>0.75</v>
+      </c>
+      <c r="N83" s="59">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="O83" s="59" t="str">
+        <v>23</v>
+      </c>
+      <c r="O83" s="59">
         <f>IF(A83="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N83))</f>
-        <v/>
+        <v>-3</v>
       </c>
     </row>
     <row r="84" spans="1:15" ht="54" customHeight="1">
-      <c r="A84" s="54"/>
-      <c r="B84" s="13"/>
+      <c r="A84" s="54">
+        <v>46220</v>
+      </c>
+      <c r="B84" s="13" t="s">
+        <v>50</v>
+      </c>
       <c r="C84" s="13"/>
-      <c r="D84" s="13"/>
-      <c r="E84" s="46"/>
-      <c r="F84" s="46" t="str">
+      <c r="D84" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="E84" s="46">
+        <v>1.25</v>
+      </c>
+      <c r="F84" s="46">
         <f>IF(A84="","",Einstellungen!$B$5)</f>
-        <v/>
-      </c>
-      <c r="G84" s="47" t="str">
+        <v>85</v>
+      </c>
+      <c r="G84" s="47">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H84" s="14" t="str">
+        <v>0</v>
+      </c>
+      <c r="H84" s="14">
         <f t="shared" si="8"/>
-        <v/>
+        <v>29</v>
       </c>
       <c r="I84" s="13" t="str">
         <f t="shared" si="6"/>
-        <v/>
+        <v>Juli YYYY</v>
       </c>
       <c r="J84" s="13"/>
       <c r="K84" s="13"/>
-      <c r="L84" s="59" t="str">
+      <c r="L84" s="59">
         <f>IF(A84="","",IF(Einstellungen!$B$15="","",MAX(0,MIN(E84,Einstellungen!$B$15-(SUMIFS($E$13:$E84,$H$13:$H84,H84)-E84)))))</f>
-        <v/>
-      </c>
-      <c r="M84" s="59" t="str">
+        <v>0</v>
+      </c>
+      <c r="M84" s="59">
         <f t="shared" si="9"/>
-        <v/>
-      </c>
-      <c r="N84" s="59" t="str">
+        <v>1.25</v>
+      </c>
+      <c r="N84" s="59">
         <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="O84" s="59" t="str">
+        <v>23</v>
+      </c>
+      <c r="O84" s="59">
         <f>IF(A84="","",IF(Einstellungen!$B$15="","",Einstellungen!$B$15-N84))</f>
-        <v/>
+        <v>-3</v>
       </c>
     </row>
     <row r="85" spans="1:15" ht="54" customHeight="1">

</xml_diff>